<commit_message>
Practicing IFS | Logical function
</commit_message>
<xml_diff>
--- a/2_Formulas_Functions/3_Logical_Functions.xlsx
+++ b/2_Formulas_Functions/3_Logical_Functions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7456b23f02075ab8/Documents/Excel LUKE/2_Formulas_Functions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="60" documentId="8_{F149B6F7-FF49-4A96-AFFD-8D9FF3E14A5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39E7CA80-A35D-4504-B86A-DCABECE69288}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="8_{F149B6F7-FF49-4A96-AFFD-8D9FF3E14A5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C5A1671-FA82-46C5-83F1-9B24B692F44A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{F15A0433-EE71-44AF-AD89-1150CA7AD24B}"/>
   </bookViews>
@@ -818,6 +818,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2016,7 +2020,7 @@
         <v>56</v>
       </c>
       <c r="K3" t="str">
-        <f t="shared" ref="K2:L21" si="0">IF($A3=K$1,"Desired", "Not Desired")</f>
+        <f t="shared" ref="K3:L21" si="0">IF($A3=K$1,"Desired", "Not Desired")</f>
         <v>Desired</v>
       </c>
       <c r="L3" t="str">

</xml_diff>